<commit_message>
session 29/07: DAILY xlsx row 31 TAG+BR, fn=1 marks, BLUAI label, OI trace scripts
- CASE_TAG.xlsx DAILY row 31 (2026-07-29): B=0.001215, L=11172261, O/P/Q/formulas; comments Q30/Q31/I30 fn=1 low_conf
- CASE_BR.xlsx row 67: G/H/I funding fields; comments Q67/I67 fn=1 low_conf
- CLAUDE.md: quy ước Zone-A-fallback khi fn=1, cấm CSV trong docs/case_files/
- cooldown_review: sửa nhãn BLUAI gLSR 2.53 = crowd long dày = wrong-side (không phải tier A hot)
- probe scripts: _probe_p1_verify, _remote_oi_trace, _remote_oi2, _run_oi_trace (BR OI provenance)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BR.xlsx
+++ b/docs/case_files/CASE_BR.xlsx
@@ -458,6 +458,26 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>agent</author>
+  </authors>
+  <commentList>
+    <comment ref="I67" authorId="0" shapeId="0">
+      <text>
+        <t>fn=1: only 1 funding snapshot for Jul29 (native_1d low_conf)</t>
+      </text>
+    </comment>
+    <comment ref="Q67" authorId="0" shapeId="0">
+      <text>
+        <t>fn=1 low_conf: single 1d snapshot (native_1d). Export lsr_global_r=1.9438 matches.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -5499,13 +5519,13 @@
       <c r="F67" s="33" t="n">
         <v>0.00018</v>
       </c>
-      <c r="G67" t="n">
+      <c r="G67" s="33" t="n">
         <v>0.00017978</v>
       </c>
-      <c r="H67" t="n">
+      <c r="H67" s="33" t="n">
         <v>0.00017978</v>
       </c>
-      <c r="I67" t="n">
+      <c r="I67" s="33" t="n">
         <v>1</v>
       </c>
       <c r="J67" s="33" t="inlineStr">
@@ -5596,6 +5616,7 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
case_daily 2.1+2.5(a): alert index-logic taker-writer + taker convert TAG/BR
- 2.1(a): telegram_error trước raise Exit(1) khi CSV abort
- 2.1(b): _load_index nhận log param, REGISTERED-NOT-OPEN INFO skip
- 2.1b-bổ-sung: orphan case file → WARNING; missing xlsx → ERROR+ping+exit
- 2.5(a): _append_daily_row col 5 × 100 (fraction→percent khi ghi)
- whale_collector/alert.py: telegram_error dedup 60s, log.error khi thiếu creds
- CASE_BR DAILY: 61 cells taker fraction→percent (26/05–28/07+08/05)
- CASE_TAG DAILY: 6 cells taker fraction→percent (29/07–03/08)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BR.xlsx
+++ b/docs/case_files/CASE_BR.xlsx
@@ -793,7 +793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AO69"/>
+  <dimension ref="A1:AO70"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="33" min="1" max="1"/>
@@ -1072,7 +1072,7 @@
         <v>2600000</v>
       </c>
       <c r="E3" s="33" t="n">
-        <v>0.4934</v>
+        <v>49.34</v>
       </c>
       <c r="F3" s="33" t="n">
         <v>0.000109765</v>
@@ -1162,7 +1162,7 @@
         <v>3000000</v>
       </c>
       <c r="E4" s="33" t="n">
-        <v>0.4906</v>
+        <v>49.06</v>
       </c>
       <c r="F4" s="33" t="n">
         <v>5e-05</v>
@@ -1252,7 +1252,7 @@
         <v>4400000</v>
       </c>
       <c r="E5" s="33" t="n">
-        <v>0.4432</v>
+        <v>44.32</v>
       </c>
       <c r="F5" s="33" t="n">
         <v>5e-05</v>
@@ -1342,7 +1342,7 @@
         <v>1500000</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>0.4816</v>
+        <v>48.16</v>
       </c>
       <c r="F6" s="33" t="n">
         <v>5e-05</v>
@@ -1413,7 +1413,7 @@
         <v>900000</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>0.4797</v>
+        <v>47.97</v>
       </c>
       <c r="F7" s="33" t="n">
         <v>0.00011623333</v>
@@ -1503,7 +1503,7 @@
         <v>940000</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>0.5222</v>
+        <v>52.22</v>
       </c>
       <c r="F8" s="57" t="n">
         <v>0.00018228333</v>
@@ -1580,7 +1580,7 @@
         <v>1700000</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>0.4631</v>
+        <v>46.31</v>
       </c>
       <c r="F9" s="33" t="n">
         <v>0.00020909667</v>
@@ -1648,7 +1648,7 @@
         <v>1600000</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>0.4576</v>
+        <v>45.76</v>
       </c>
       <c r="F10" s="33" t="n">
         <v>6.944e-05</v>
@@ -1716,7 +1716,7 @@
         <v>5800000</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>0.4533</v>
+        <v>45.33</v>
       </c>
       <c r="F11" s="33" t="n">
         <v>0.00031061</v>
@@ -1784,7 +1784,7 @@
         <v>3800000</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>0.5031</v>
+        <v>50.31</v>
       </c>
       <c r="F12" s="33" t="n">
         <v>5e-05</v>
@@ -1852,7 +1852,7 @@
         <v>2400000</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>0.4977</v>
+        <v>49.77</v>
       </c>
       <c r="F13" s="33" t="n">
         <v>5e-05</v>
@@ -1920,7 +1920,7 @@
         <v>1400000</v>
       </c>
       <c r="E14" s="33" t="n">
-        <v>0.4735</v>
+        <v>47.35</v>
       </c>
       <c r="F14" s="33" t="n">
         <v>5e-05</v>
@@ -1988,7 +1988,7 @@
         <v>3100000</v>
       </c>
       <c r="E15" s="33" t="n">
-        <v>0.4691</v>
+        <v>46.91</v>
       </c>
       <c r="F15" s="33" t="n">
         <v>7.9311667e-05</v>
@@ -2056,7 +2056,7 @@
         <v>1300000</v>
       </c>
       <c r="E16" s="33" t="n">
-        <v>0.4694</v>
+        <v>46.94</v>
       </c>
       <c r="F16" s="33" t="n">
         <v>8.053333299999999e-05</v>
@@ -2124,7 +2124,7 @@
         <v>1400000</v>
       </c>
       <c r="E17" s="33" t="n">
-        <v>0.456</v>
+        <v>45.6</v>
       </c>
       <c r="F17" s="33" t="n">
         <v>0.00013595333</v>
@@ -2192,7 +2192,7 @@
         <v>2800000</v>
       </c>
       <c r="E18" s="33" t="n">
-        <v>0.4918</v>
+        <v>49.18</v>
       </c>
       <c r="F18" s="33" t="n">
         <v>0.000173085</v>
@@ -2260,7 +2260,7 @@
         <v>8800000</v>
       </c>
       <c r="E19" s="33" t="n">
-        <v>0.4639</v>
+        <v>46.39</v>
       </c>
       <c r="F19" s="33" t="n">
         <v>5.274e-05</v>
@@ -2328,7 +2328,7 @@
         <v>3200000</v>
       </c>
       <c r="E20" s="33" t="n">
-        <v>0.4594</v>
+        <v>45.94</v>
       </c>
       <c r="F20" s="33" t="n">
         <v>5.4401667e-05</v>
@@ -2396,7 +2396,7 @@
         <v>1900000</v>
       </c>
       <c r="E21" s="33" t="n">
-        <v>0.465</v>
+        <v>46.5</v>
       </c>
       <c r="F21" s="33" t="n">
         <v>5e-05</v>
@@ -2464,7 +2464,7 @@
         <v>890000</v>
       </c>
       <c r="E22" s="33" t="n">
-        <v>0.4763</v>
+        <v>47.63</v>
       </c>
       <c r="F22" s="33" t="n">
         <v>5e-05</v>
@@ -2532,7 +2532,7 @@
         <v>990000</v>
       </c>
       <c r="E23" s="33" t="n">
-        <v>0.4919</v>
+        <v>49.19</v>
       </c>
       <c r="F23" s="33" t="n">
         <v>8.4536667e-05</v>
@@ -2600,7 +2600,7 @@
         <v>130000000</v>
       </c>
       <c r="E24" s="33" t="n">
-        <v>0.5155999999999999</v>
+        <v>51.56</v>
       </c>
       <c r="F24" s="33" t="n">
         <v>0.00026853</v>
@@ -2668,7 +2668,7 @@
         <v>160000000</v>
       </c>
       <c r="E25" s="33" t="n">
-        <v>0.5208</v>
+        <v>52.08</v>
       </c>
       <c r="F25" s="33" t="n">
         <v>0.00018252</v>
@@ -2736,7 +2736,7 @@
         <v>32000000</v>
       </c>
       <c r="E26" s="33" t="n">
-        <v>0.5115</v>
+        <v>51.15</v>
       </c>
       <c r="F26" s="33" t="n">
         <v>0.00019495167</v>
@@ -2804,7 +2804,7 @@
         <v>9100000</v>
       </c>
       <c r="E27" s="33" t="n">
-        <v>0.5219</v>
+        <v>52.19</v>
       </c>
       <c r="F27" s="33" t="n">
         <v>8.0766667e-05</v>
@@ -2872,7 +2872,7 @@
         <v>2900000</v>
       </c>
       <c r="E28" s="33" t="n">
-        <v>0.539</v>
+        <v>53.9</v>
       </c>
       <c r="F28" s="33" t="n">
         <v>5e-05</v>
@@ -2940,7 +2940,7 @@
         <v>3900000</v>
       </c>
       <c r="E29" s="33" t="n">
-        <v>0.5097</v>
+        <v>50.97</v>
       </c>
       <c r="F29" s="33" t="n">
         <v>8.828666700000001e-05</v>
@@ -3008,7 +3008,7 @@
         <v>3100000</v>
       </c>
       <c r="E30" s="33" t="n">
-        <v>0.4863</v>
+        <v>48.63</v>
       </c>
       <c r="F30" s="33" t="n">
         <v>8.498666699999999e-05</v>
@@ -3076,7 +3076,7 @@
         <v>24000000</v>
       </c>
       <c r="E31" s="33" t="n">
-        <v>0.4965</v>
+        <v>49.65</v>
       </c>
       <c r="F31" s="33" t="n">
         <v>0.00020984333</v>
@@ -3144,7 +3144,7 @@
         <v>11000000</v>
       </c>
       <c r="E32" s="33" t="n">
-        <v>0.4897</v>
+        <v>48.97</v>
       </c>
       <c r="F32" s="33" t="n">
         <v>0.00010257</v>
@@ -3212,7 +3212,7 @@
         <v>3700000</v>
       </c>
       <c r="E33" s="33" t="n">
-        <v>0.4943</v>
+        <v>49.43</v>
       </c>
       <c r="F33" s="33" t="n">
         <v>5e-05</v>
@@ -3280,7 +3280,7 @@
         <v>2600000</v>
       </c>
       <c r="E34" s="33" t="n">
-        <v>0.4794</v>
+        <v>47.94</v>
       </c>
       <c r="F34" s="33" t="n">
         <v>5e-05</v>
@@ -3348,7 +3348,7 @@
         <v>9600000</v>
       </c>
       <c r="E35" s="33" t="n">
-        <v>0.4935</v>
+        <v>49.35</v>
       </c>
       <c r="F35" s="33" t="n">
         <v>5.0966667e-05</v>
@@ -3416,7 +3416,7 @@
         <v>7800000</v>
       </c>
       <c r="E36" s="33" t="n">
-        <v>0.4773</v>
+        <v>47.73</v>
       </c>
       <c r="F36" s="33" t="n">
         <v>5e-05</v>
@@ -3484,7 +3484,7 @@
         <v>10000000</v>
       </c>
       <c r="E37" s="33" t="n">
-        <v>0.4991</v>
+        <v>49.91</v>
       </c>
       <c r="F37" s="33" t="n">
         <v>5.3536667e-05</v>
@@ -3552,7 +3552,7 @@
         <v>3900000</v>
       </c>
       <c r="E38" s="33" t="n">
-        <v>0.5014</v>
+        <v>50.14</v>
       </c>
       <c r="F38" s="33" t="n">
         <v>6.0115e-05</v>
@@ -3620,7 +3620,7 @@
         <v>3700000</v>
       </c>
       <c r="E39" s="33" t="n">
-        <v>0.4994</v>
+        <v>49.94</v>
       </c>
       <c r="F39" s="33" t="n">
         <v>6.6176667e-05</v>
@@ -3688,7 +3688,7 @@
         <v>4700000</v>
       </c>
       <c r="E40" s="33" t="n">
-        <v>0.4888</v>
+        <v>48.88</v>
       </c>
       <c r="F40" s="33" t="n">
         <v>5.2778333e-05</v>
@@ -3756,7 +3756,7 @@
         <v>3600000</v>
       </c>
       <c r="E41" s="33" t="n">
-        <v>0.4717</v>
+        <v>47.17</v>
       </c>
       <c r="F41" s="33" t="n">
         <v>9.3916667e-05</v>
@@ -3824,7 +3824,7 @@
         <v>2400000</v>
       </c>
       <c r="E42" s="33" t="n">
-        <v>0.4882</v>
+        <v>48.82</v>
       </c>
       <c r="F42" s="33" t="n">
         <v>6.4121667e-05</v>
@@ -3892,7 +3892,7 @@
         <v>1800000</v>
       </c>
       <c r="E43" s="33" t="n">
-        <v>0.4838</v>
+        <v>48.38</v>
       </c>
       <c r="F43" s="33" t="n">
         <v>6.1806667e-05</v>
@@ -3960,7 +3960,7 @@
         <v>3100000</v>
       </c>
       <c r="E44" s="33" t="n">
-        <v>0.4586</v>
+        <v>45.86</v>
       </c>
       <c r="F44" s="33" t="n">
         <v>0.000159465</v>
@@ -4028,7 +4028,7 @@
         <v>3100000</v>
       </c>
       <c r="E45" s="33" t="n">
-        <v>0.4882</v>
+        <v>48.82</v>
       </c>
       <c r="F45" s="33" t="n">
         <v>5.0818333e-05</v>
@@ -4096,7 +4096,7 @@
         <v>2900000</v>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.5201</v>
+        <v>52.01</v>
       </c>
       <c r="F46" s="33" t="n">
         <v>5.9325e-05</v>
@@ -4164,7 +4164,7 @@
         <v>1800000</v>
       </c>
       <c r="E47" s="33" t="n">
-        <v>0.5019</v>
+        <v>50.19</v>
       </c>
       <c r="F47" s="33" t="n">
         <v>0.00011703333</v>
@@ -4232,7 +4232,7 @@
         <v>1700000</v>
       </c>
       <c r="E48" s="33" t="n">
-        <v>0.524</v>
+        <v>52.4</v>
       </c>
       <c r="F48" s="33" t="n">
         <v>0.00027251833</v>
@@ -4300,7 +4300,7 @@
         <v>1700000</v>
       </c>
       <c r="E49" s="33" t="n">
-        <v>0.4459</v>
+        <v>44.59</v>
       </c>
       <c r="F49" s="33" t="n">
         <v>0.00011145167</v>
@@ -4368,7 +4368,7 @@
         <v>1300000</v>
       </c>
       <c r="E50" s="33" t="n">
-        <v>0.4889</v>
+        <v>48.89</v>
       </c>
       <c r="F50" s="33" t="n">
         <v>7.4968333e-05</v>
@@ -4436,7 +4436,7 @@
         <v>1300000</v>
       </c>
       <c r="E51" s="33" t="n">
-        <v>0.53</v>
+        <v>53</v>
       </c>
       <c r="F51" s="33" t="n">
         <v>7.6065e-05</v>
@@ -4504,7 +4504,7 @@
         <v>1700000</v>
       </c>
       <c r="E52" s="33" t="n">
-        <v>0.5206</v>
+        <v>52.06</v>
       </c>
       <c r="F52" s="33" t="n">
         <v>0.00018826333</v>
@@ -4572,7 +4572,7 @@
         <v>1900000</v>
       </c>
       <c r="E53" s="33" t="n">
-        <v>0.4893</v>
+        <v>48.93</v>
       </c>
       <c r="F53" s="33" t="n">
         <v>6.2358333e-05</v>
@@ -4640,7 +4640,7 @@
         <v>1500000</v>
       </c>
       <c r="E54" s="33" t="n">
-        <v>0.4831</v>
+        <v>48.31</v>
       </c>
       <c r="F54" s="33" t="n">
         <v>0.00015960333</v>
@@ -4708,7 +4708,7 @@
         <v>1900000</v>
       </c>
       <c r="E55" s="33" t="n">
-        <v>0.5207000000000001</v>
+        <v>52.07</v>
       </c>
       <c r="F55" s="33" t="n">
         <v>0.000134</v>
@@ -4776,7 +4776,7 @@
         <v>5300000</v>
       </c>
       <c r="E56" s="33" t="n">
-        <v>0.4746</v>
+        <v>47.46</v>
       </c>
       <c r="F56" s="33" t="n">
         <v>0.00010645333</v>
@@ -4844,7 +4844,7 @@
         <v>6000000</v>
       </c>
       <c r="E57" s="33" t="n">
-        <v>0.4506</v>
+        <v>45.06</v>
       </c>
       <c r="F57" s="33" t="n">
         <v>7.808e-05</v>
@@ -4912,7 +4912,7 @@
         <v>2300000</v>
       </c>
       <c r="E58" s="33" t="n">
-        <v>0.4777</v>
+        <v>47.77</v>
       </c>
       <c r="F58" s="33" t="n">
         <v>5e-05</v>
@@ -4980,7 +4980,7 @@
         <v>3000000</v>
       </c>
       <c r="E59" s="33" t="n">
-        <v>0.5315</v>
+        <v>53.15</v>
       </c>
       <c r="F59" s="33" t="n">
         <v>5e-05</v>
@@ -5048,7 +5048,7 @@
         <v>5300000</v>
       </c>
       <c r="E60" s="33" t="n">
-        <v>0.4714</v>
+        <v>47.14</v>
       </c>
       <c r="F60" s="33" t="n">
         <v>5.7938333e-05</v>
@@ -5116,7 +5116,7 @@
         <v>6500000</v>
       </c>
       <c r="E61" s="33" t="n">
-        <v>0.4939</v>
+        <v>49.39</v>
       </c>
       <c r="F61" s="33" t="n">
         <v>5e-05</v>
@@ -5457,7 +5457,7 @@
         <v>604348.24303</v>
       </c>
       <c r="E66" s="33" t="n">
-        <v>0.50852705558559</v>
+        <v>50.852706</v>
       </c>
       <c r="F66" s="33" t="n">
         <v>7.913499999999999e-05</v>
@@ -5527,7 +5527,7 @@
         <v>667504.9977000001</v>
       </c>
       <c r="E67" s="33" t="n">
-        <v>0.4817578772802653</v>
+        <v>48.175788</v>
       </c>
       <c r="F67" s="33" t="n">
         <v>0.0001180016666666</v>
@@ -5604,7 +5604,7 @@
         <v>670325.09431</v>
       </c>
       <c r="E68" s="33" t="n">
-        <v>0.4917407878017789</v>
+        <v>49.174079</v>
       </c>
       <c r="F68" s="33" t="n">
         <v>5e-05</v>
@@ -5656,70 +5656,138 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="33" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="B69" t="n">
+      <c r="B69" s="33" t="n">
         <v>0.1503439699877407</v>
       </c>
-      <c r="C69">
+      <c r="C69" s="33">
         <f>IFERROR(B69/B68-1,"")</f>
         <v/>
       </c>
-      <c r="D69" t="n">
+      <c r="D69" s="33" t="n">
         <v>618332.5749499999</v>
       </c>
-      <c r="E69" t="n">
-        <v>0.4643813604713444</v>
-      </c>
-      <c r="F69" t="n">
+      <c r="E69" s="33" t="n">
+        <v>46.438136</v>
+      </c>
+      <c r="F69" s="33" t="n">
         <v>9.5085e-05</v>
       </c>
-      <c r="G69" t="n">
-        <v>5e-05</v>
-      </c>
-      <c r="H69" t="n">
+      <c r="G69" s="33" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="H69" s="33" t="n">
         <v>0.00015113</v>
       </c>
-      <c r="I69" t="n">
+      <c r="I69" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="L69" t="n">
+      <c r="L69" s="33" t="n">
         <v>3840661.32366</v>
       </c>
-      <c r="O69" t="n">
+      <c r="O69" s="33" t="n">
         <v>1.6509</v>
       </c>
-      <c r="P69" t="n">
+      <c r="P69" s="33" t="n">
         <v>1.3998</v>
       </c>
-      <c r="Q69" t="n">
+      <c r="Q69" s="33" t="n">
         <v>1.8401</v>
       </c>
-      <c r="R69">
+      <c r="R69" s="33">
         <f>IFERROR(O69/P69,"")</f>
         <v/>
       </c>
-      <c r="S69">
+      <c r="S69" s="33">
         <f>IFERROR(AVERAGE(R67:R69),"")</f>
         <v/>
       </c>
-      <c r="T69">
+      <c r="T69" s="33">
         <f>IFERROR(Q69/Q64,"")</f>
         <v/>
       </c>
-      <c r="U69">
+      <c r="U69" s="33">
         <f>IFERROR(O69/O66-1,"")</f>
         <v/>
       </c>
-      <c r="V69">
+      <c r="V69" s="33">
         <f>IFERROR(P69/P66-1,"")</f>
         <v/>
       </c>
-      <c r="AJ69">
+      <c r="AJ69" s="33">
         <f>IF(OR(AB69="",D69="",D69=0),"",AB69/D69)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="33" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B70" s="33" t="n">
+        <v>0.1437135231999385</v>
+      </c>
+      <c r="C70" s="33">
+        <f>IFERROR(B70/B69-1,"")</f>
+        <v/>
+      </c>
+      <c r="D70" s="33" t="n">
+        <v>591029.62469</v>
+      </c>
+      <c r="E70" s="33" t="n">
+        <v>49.315763</v>
+      </c>
+      <c r="F70" s="33" t="n">
+        <v>0.0004032633333333334</v>
+      </c>
+      <c r="G70" s="33" t="n">
+        <v>0.00032365</v>
+      </c>
+      <c r="H70" s="33" t="n">
+        <v>0.00059693</v>
+      </c>
+      <c r="I70" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="L70" s="33" t="n">
+        <v>3623386.30443</v>
+      </c>
+      <c r="O70" s="33" t="n">
+        <v>1.7023</v>
+      </c>
+      <c r="P70" s="33" t="n">
+        <v>1.3613</v>
+      </c>
+      <c r="Q70" s="33" t="n">
+        <v>1.7196</v>
+      </c>
+      <c r="R70" s="33">
+        <f>IFERROR(O70/P70,"")</f>
+        <v/>
+      </c>
+      <c r="S70" s="33">
+        <f>IFERROR(AVERAGE(R68:R70),"")</f>
+        <v/>
+      </c>
+      <c r="T70" s="33">
+        <f>IFERROR(Q70/Q65,"")</f>
+        <v/>
+      </c>
+      <c r="U70" s="33">
+        <f>IFERROR(O70/O67-1,"")</f>
+        <v/>
+      </c>
+      <c r="V70" s="33">
+        <f>IFERROR(P70/P67-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ70" s="33">
+        <f>IF(OR(AB70="",D70="",D70=0),"",AB70/D70)</f>
         <v/>
       </c>
     </row>

</xml_diff>